<commit_message>
feat(costs): add CAPEX annualization (CRF) and FACTS sizing cost
- Add discount rate + useful lives params (CREG WACC 11.5%, lives)
- Annualize line/BESS/FACTS investments via capital recovery factor
- Add FACTS sizing cost Cf_size*|dB_f| with dB_abs + linearization
- Compute per-line TCSC compensation range from line reactance
</commit_message>
<xml_diff>
--- a/01_Data/03_Test_Cases/caso_IEEE6_ww.xlsx
+++ b/01_Data/03_Test_Cases/caso_IEEE6_ww.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\2. Universidad Nacional de Colombia\2. Postgraduate\1_SEMESTER\TESIS DE MAESTRIA\2nd Search\04_TESIS_DANIEL\03_CODIGO_TRABAJO_DANIEL\BESS_FACTS_master\01_Data\03_Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51C87F6D-DC98-4A14-AAE6-09B87A21AF61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{006C0123-9D33-4BA3-B22F-77EF3B3F193F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCCIONES" sheetId="1" r:id="rId1"/>
@@ -25,8 +25,40 @@
     <sheet name="FACTS_Cand" sheetId="10" r:id="rId10"/>
     <sheet name="Demanda" sheetId="11" r:id="rId11"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={52E7122E-D638-4998-B53F-C7119B19FE0A}</author>
+  </authors>
+  <commentList>
+    <comment ref="B6" authorId="0" shapeId="0" xr:uid="{52E7122E-D638-4998-B53F-C7119B19FE0A}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Se puso 70 en todos los nodos para poder hacer las validaciones AC con el modelo de matpower
+Antes era 42.5 para todos los nodos</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -423,7 +455,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -473,6 +505,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -527,7 +565,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -543,7 +581,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -567,6 +604,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Daniel Lindo" id="{34EE5DEF-6423-48EB-AACB-BA92017EBEB5}" userId="S::dalindop@unal.edu.co::bac517a2-50e1-4afb-8365-3aec15672be1" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -852,6 +895,15 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="B6" dT="2026-07-13T00:28:30.94" personId="{34EE5DEF-6423-48EB-AACB-BA92017EBEB5}" id="{52E7122E-D638-4998-B53F-C7119B19FE0A}">
+    <text>Se puso 70 en todos los nodos para poder hacer las validaciones AC con el modelo de matpower
+Antes era 42.5 para todos los nodos</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A26"/>
@@ -971,7 +1023,7 @@
       <c r="A25" s="2"/>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1030,7 +1082,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:D29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1078,13 +1130,13 @@
         <v>1</v>
       </c>
       <c r="B6" s="5">
-        <v>42.5</v>
+        <v>70</v>
       </c>
       <c r="C6" s="5">
-        <v>42.5</v>
+        <v>70</v>
       </c>
       <c r="D6" s="5">
-        <v>42.5</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1411,6 +1463,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1454,7 +1507,7 @@
       <c r="A6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="7">
         <v>100</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1465,7 +1518,7 @@
       <c r="A7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="7">
         <v>24</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -1476,7 +1529,7 @@
       <c r="A8" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="8">
         <v>3</v>
       </c>
       <c r="C8" s="6" t="s">
@@ -1487,7 +1540,7 @@
       <c r="A9" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="8">
         <v>3</v>
       </c>
       <c r="C9" s="6" t="s">
@@ -1498,7 +1551,7 @@
       <c r="A10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="8">
         <v>0.01</v>
       </c>
       <c r="C10" s="6" t="s">
@@ -1509,7 +1562,7 @@
       <c r="A11" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="8">
         <v>1800</v>
       </c>
       <c r="C11" s="6" t="s">
@@ -2081,7 +2134,7 @@
       <c r="D6" s="5">
         <v>200</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="8">
         <v>200</v>
       </c>
       <c r="F6" s="5">
@@ -2093,16 +2146,16 @@
       <c r="H6" s="5">
         <v>213.1</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="8">
         <v>1</v>
       </c>
-      <c r="J6" s="9">
+      <c r="J6" s="8">
         <v>1</v>
       </c>
-      <c r="K6" s="9">
+      <c r="K6" s="8">
         <v>0</v>
       </c>
-      <c r="L6" s="9">
+      <c r="L6" s="8">
         <v>0</v>
       </c>
     </row>
@@ -2119,7 +2172,7 @@
       <c r="D7" s="5">
         <v>150</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="8">
         <v>150</v>
       </c>
       <c r="F7" s="5">
@@ -2131,16 +2184,16 @@
       <c r="H7" s="5">
         <v>200</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="8">
         <v>1</v>
       </c>
-      <c r="J7" s="9">
+      <c r="J7" s="8">
         <v>1</v>
       </c>
-      <c r="K7" s="9">
+      <c r="K7" s="8">
         <v>0</v>
       </c>
-      <c r="L7" s="9">
+      <c r="L7" s="8">
         <v>0</v>
       </c>
     </row>
@@ -2157,7 +2210,7 @@
       <c r="D8" s="5">
         <v>180</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="8">
         <v>180</v>
       </c>
       <c r="F8" s="5">
@@ -2169,16 +2222,16 @@
       <c r="H8" s="5">
         <v>240</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I8" s="8">
         <v>1</v>
       </c>
-      <c r="J8" s="9">
+      <c r="J8" s="8">
         <v>1</v>
       </c>
-      <c r="K8" s="9">
+      <c r="K8" s="8">
         <v>0</v>
       </c>
-      <c r="L8" s="9">
+      <c r="L8" s="8">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(cases): Test the cases with IEEE 6
</commit_message>
<xml_diff>
--- a/01_Data/03_Test_Cases/caso_IEEE6_ww.xlsx
+++ b/01_Data/03_Test_Cases/caso_IEEE6_ww.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\2. Universidad Nacional de Colombia\2. Postgraduate\1_SEMESTER\TESIS DE MAESTRIA\2nd Search\04_TESIS_DANIEL\03_CODIGO_TRABAJO_DANIEL\BESS_FACTS_master\01_Data\03_Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{006C0123-9D33-4BA3-B22F-77EF3B3F193F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1342A91-1D1B-47C2-8742-9377825D1E6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCCIONES" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="130">
   <si>
     <t>Plantilla de datos - Modelo TEP con BESS y FACTS</t>
   </si>
@@ -449,13 +449,16 @@
   </si>
   <si>
     <t>UNIDADES: indicadas en la fila bajo cada encabezado. (No borrarlas ni modificarlas)</t>
+  </si>
+  <si>
+    <t>rundcpf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -505,12 +508,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1685,7 +1682,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="6" width="16" customWidth="1"/>
@@ -1957,6 +1954,11 @@
       </c>
       <c r="F16" s="5">
         <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="10:10" x14ac:dyDescent="0.25">
+      <c r="J17" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>